<commit_message>
Making temperature day plotting python file
C
</commit_message>
<xml_diff>
--- a/BeatnotePostCombFix/Apr06,2026/Aril6.xlsx
+++ b/BeatnotePostCombFix/Apr06,2026/Aril6.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\BeatnotePostCombFix\Apr06,2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostCombFix\Apr06,2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F58C326-A76F-4D34-999B-8C378D00F166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3938FF82-48EB-426B-8C9C-295C91E714DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{DE27D4D9-8A5E-4A81-9645-FB782B2C9508}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DE27D4D9-8A5E-4A81-9645-FB782B2C9508}"/>
   </bookViews>
   <sheets>
     <sheet name="456" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="894" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,16 +28,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -116,12 +117,21 @@
   <si>
     <t>Apr06,2026+6-03-01PM</t>
   </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>std</t>
+  </si>
+  <si>
+    <t>%std/mean</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -472,7 +482,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -480,6 +489,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -591,7 +601,7 @@
           </c:marker>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet2!$B$2:$B$15</c:f>
+              <c:f>'894'!$B$2:$B$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -791,7 +801,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -799,6 +808,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1949,16 +1959,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>536575</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>381000</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>403882</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>261772</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>231775</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>361950</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>162582</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>337973</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1990,16 +2000,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>244475</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>368300</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>282575</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>358775</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>549275</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>349250</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>53975</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>339725</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2344,10 +2354,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E67E67-BE51-40B6-BF6A-AB076C1A076C}">
-  <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:Q19"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="10" max="10" width="10.375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2373,7 +2386,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -2398,8 +2411,29 @@
       <c r="H2" s="1">
         <v>6.7331913797042502E-3</v>
       </c>
+      <c r="K2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="42.75">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -2423,17 +2457,40 @@
       </c>
       <c r="H3" s="1">
         <v>7.4830854729079901E-3</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
       </c>
       <c r="K3">
         <f>AVERAGE(B2:B19)</f>
         <v>0.20333642314313793</v>
       </c>
       <c r="L3">
-        <f>K4/K3</f>
-        <v>1.2794565494556256E-2</v>
+        <f>AVERAGE(C2:C19)</f>
+        <v>1.331004147377965</v>
+      </c>
+      <c r="M3">
+        <f>AVERAGE(D2:D19)</f>
+        <v>-1.343352237272212E-3</v>
+      </c>
+      <c r="N3">
+        <f>AVERAGE(E2:E19)</f>
+        <v>2.3941378865325134</v>
+      </c>
+      <c r="O3">
+        <f>AVERAGE(F2:F19)</f>
+        <v>41.727967895474265</v>
+      </c>
+      <c r="P3">
+        <f>AVERAGE(G2:G19)</f>
+        <v>8.9884161107294783E-4</v>
+      </c>
+      <c r="Q3">
+        <f>AVERAGE(H2:H19)</f>
+        <v>6.7196783564735787E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" ht="42.75">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -2457,13 +2514,40 @@
       </c>
       <c r="H4" s="1">
         <v>6.8554338102289102E-3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>27</v>
       </c>
       <c r="K4">
         <f>_xlfn.STDEV.S(B2:B19)</f>
         <v>2.6016011833336827E-3</v>
       </c>
+      <c r="L4">
+        <f>_xlfn.STDEV.S(C2:C19)</f>
+        <v>1.3813454075544782E-3</v>
+      </c>
+      <c r="M4">
+        <f>_xlfn.STDEV.S(D2:D19)</f>
+        <v>2.5170715272718175E-4</v>
+      </c>
+      <c r="N4">
+        <f>_xlfn.STDEV.S(E2:E19)</f>
+        <v>0.67013895879129959</v>
+      </c>
+      <c r="O4">
+        <f>_xlfn.STDEV.S(F2:F19)</f>
+        <v>1.6798617742726416</v>
+      </c>
+      <c r="P4">
+        <f>_xlfn.STDEV.S(G2:G19)</f>
+        <v>3.2202999446943339E-4</v>
+      </c>
+      <c r="Q4">
+        <f>_xlfn.STDEV.S(H2:H19)</f>
+        <v>8.7450229714018397E-4</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" ht="42.75">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -2489,7 +2573,7 @@
         <v>6.0223458005847002E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" ht="42.75">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -2514,8 +2598,39 @@
       <c r="H6" s="1">
         <v>7.5022586093307997E-3</v>
       </c>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6">
+        <f>K4/K3*100</f>
+        <v>1.2794565494556256</v>
+      </c>
+      <c r="L6">
+        <f t="shared" ref="L6:Q6" si="0">L4/L3*100</f>
+        <v>0.1037822016013762</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="0"/>
+        <v>-18.737241487630524</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="0"/>
+        <v>27.990825531017251</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="0"/>
+        <v>4.0257454628046627</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="0"/>
+        <v>35.82722367348191</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="0"/>
+        <v>13.014049940317593</v>
+      </c>
     </row>
-    <row r="7" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" ht="42.75">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -2540,8 +2655,12 @@
       <c r="H7" s="1">
         <v>5.4512116460360199E-3</v>
       </c>
+      <c r="K7">
+        <f>K6/SQRT(18*8)</f>
+        <v>0.10662137912130214</v>
+      </c>
     </row>
-    <row r="8" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" ht="42.75">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -2567,7 +2686,7 @@
         <v>7.7968480004249902E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" ht="42.75">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -2593,7 +2712,7 @@
         <v>7.8251933969995194E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" ht="42.75">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -2619,7 +2738,7 @@
         <v>5.6124292572678298E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" ht="42.75">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -2645,7 +2764,7 @@
         <v>7.8000210714507601E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" ht="42.75">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -2671,7 +2790,7 @@
         <v>6.9099970499809198E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" ht="42.75">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -2697,7 +2816,7 @@
         <v>6.3546524311469798E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" ht="42.75">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -2723,7 +2842,7 @@
         <v>6.5441406276150402E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" ht="42.75">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -2749,7 +2868,7 @@
         <v>7.1700855339725299E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" ht="42.75">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -2775,7 +2894,7 @@
         <v>6.5440924461874902E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="42.75">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -2801,7 +2920,7 @@
         <v>5.3561065570487502E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="42.75">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -2827,7 +2946,7 @@
         <v>7.6197773041926601E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="42.75">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -2861,10 +2980,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6499FFC7-3DA5-4057-863B-C101A2BD7DDC}">
-  <dimension ref="A1:L15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:Q15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="10" max="10" width="11" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2890,7 +3012,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -2915,16 +3037,29 @@
       <c r="H2" s="1">
         <v>3.9208188938186297E-2</v>
       </c>
-      <c r="K2">
-        <f>AVERAGE(B2:B6,B9:B15)</f>
-        <v>9.6338973054278512</v>
-      </c>
-      <c r="L2">
-        <f>K3/K2</f>
-        <v>4.378045472078553E-3</v>
+      <c r="K2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="42.75">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -2949,12 +3084,39 @@
       <c r="H3" s="1">
         <v>3.8679664000731799E-2</v>
       </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
       <c r="K3">
-        <f>_xlfn.STDEV.S(B2:B6,B9:B15)</f>
-        <v>4.2177640476498177E-2</v>
+        <f>AVERAGE(B2:B8,B9:B15)</f>
+        <v>9.6088335511934186</v>
+      </c>
+      <c r="L3">
+        <f t="shared" ref="L3:Q3" si="0">AVERAGE(C2:C8,C9:C15)</f>
+        <v>1.1621065158458728</v>
+      </c>
+      <c r="M3">
+        <f t="shared" si="0"/>
+        <v>-1.5775610011044422E-3</v>
+      </c>
+      <c r="N3">
+        <f t="shared" si="0"/>
+        <v>2.6608353107389324</v>
+      </c>
+      <c r="O3">
+        <f t="shared" si="0"/>
+        <v>41.906194637181123</v>
+      </c>
+      <c r="P3">
+        <f t="shared" si="0"/>
+        <v>2.2966578140585538E-3</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" si="0"/>
+        <v>3.9720000673721056E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" ht="42.75">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -2979,8 +3141,39 @@
       <c r="H4" s="1">
         <v>3.84398386419708E-2</v>
       </c>
+      <c r="J4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4">
+        <f>_xlfn.STDEV.S(B2:B8,B9:B15)</f>
+        <v>7.7668592218918517E-2</v>
+      </c>
+      <c r="L4">
+        <f>_xlfn.STDEV.S(C2:C8,C9:C15)</f>
+        <v>5.252449588536383E-3</v>
+      </c>
+      <c r="M4">
+        <f t="shared" ref="L4:Q4" si="1">_xlfn.STDEV.S(D2:D8,D9:D15)</f>
+        <v>9.143262698338931E-4</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="1"/>
+        <v>0.47761766086667917</v>
+      </c>
+      <c r="O4">
+        <f t="shared" si="1"/>
+        <v>1.0820372207622722</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="1"/>
+        <v>2.1205116713350879E-5</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" si="1"/>
+        <v>8.6279095495304925E-4</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" ht="42.75">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -3006,7 +3199,7 @@
         <v>3.8826109217313297E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" ht="42.75">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -3031,8 +3224,39 @@
       <c r="H6" s="1">
         <v>4.0985235994735802E-2</v>
       </c>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6">
+        <f>K4/K3*100</f>
+        <v>0.80830406526577903</v>
+      </c>
+      <c r="L6">
+        <f>L4/L3*100</f>
+        <v>0.45197660600958223</v>
+      </c>
+      <c r="M6">
+        <f>M4/M3*100</f>
+        <v>-57.958219631049325</v>
+      </c>
+      <c r="N6">
+        <f t="shared" ref="L6:Q6" si="2">N4/N3*100</f>
+        <v>17.949914409924205</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="2"/>
+        <v>2.582045996135947</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="2"/>
+        <v>0.92330327067218254</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="2"/>
+        <v>2.1721826292009001</v>
+      </c>
     </row>
-    <row r="7" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" ht="42.75">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -3057,8 +3281,12 @@
       <c r="H7" s="1">
         <v>3.9929122334316398E-2</v>
       </c>
+      <c r="K7">
+        <f>K6/SQRT(18)</f>
+        <v>0.19051909527002869</v>
+      </c>
     </row>
-    <row r="8" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" ht="42.75">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -3084,7 +3312,7 @@
         <v>3.84086464084595E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" ht="42.75">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -3110,7 +3338,7 @@
         <v>4.0270956489123703E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" ht="42.75">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -3136,7 +3364,7 @@
         <v>4.0877162789576302E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" ht="42.75">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -3162,7 +3390,7 @@
         <v>4.0195639460677099E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" ht="42.75">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -3188,7 +3416,7 @@
         <v>4.02841943243843E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" ht="42.75">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -3214,7 +3442,7 @@
         <v>3.9879989417801201E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" ht="42.75">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -3240,7 +3468,7 @@
         <v>3.9820041350796802E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" ht="42.75">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>

</xml_diff>